<commit_message>
Small Excel template update
</commit_message>
<xml_diff>
--- a/final_output/March Madness Preview 2026.xlsx
+++ b/final_output/March Madness Preview 2026.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Software Projects\march-madness-previewer\final_output\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2434ef0feffdd206/Documents/Personal Life/Sports/CBB/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{565DB17C-93B8-4C98-B658-D09FFBAB98ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{565DB17C-93B8-4C98-B658-D09FFBAB98ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{703C6182-25FF-456E-B447-BBC402D2D0E2}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{A5B2F9FC-FB27-41D3-9882-716C8D814AE7}"/>
   </bookViews>
@@ -1951,10 +1951,10 @@
     <t>Methodology:</t>
   </si>
   <si>
-    <t>Update team names in cells C7 &amp; C8</t>
+    <t>Updated on 3/16/2026</t>
   </si>
   <si>
-    <t>Updated on 3/16/2026</t>
+    <t>Edit team names in cells C7 &amp; C8 to generate desired matchup</t>
   </si>
 </sst>
 </file>
@@ -2420,10 +2420,10 @@
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="11" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -2950,8 +2950,8 @@
     <row r="5" spans="1:21" s="25" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="33"/>
       <c r="B5" s="33"/>
-      <c r="C5" s="65" t="s">
-        <v>636</v>
+      <c r="C5" s="64" t="s">
+        <v>635</v>
       </c>
       <c r="U5" s="26"/>
     </row>
@@ -2961,21 +2961,21 @@
       <c r="U6" s="26"/>
     </row>
     <row r="7" spans="1:21" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C7" s="64" t="s">
+      <c r="C7" s="65" t="s">
         <v>287</v>
       </c>
-      <c r="D7" s="64"/>
-      <c r="E7" s="64"/>
-      <c r="F7" s="64"/>
-      <c r="G7" s="64"/>
-      <c r="H7" s="64"/>
-      <c r="I7" s="64"/>
-      <c r="J7" s="64"/>
-      <c r="K7" s="64"/>
-      <c r="L7" s="64"/>
-      <c r="M7" s="64"/>
-      <c r="N7" s="64"/>
-      <c r="O7" s="64"/>
+      <c r="D7" s="65"/>
+      <c r="E7" s="65"/>
+      <c r="F7" s="65"/>
+      <c r="G7" s="65"/>
+      <c r="H7" s="65"/>
+      <c r="I7" s="65"/>
+      <c r="J7" s="65"/>
+      <c r="K7" s="65"/>
+      <c r="L7" s="65"/>
+      <c r="M7" s="65"/>
+      <c r="N7" s="65"/>
+      <c r="O7" s="65"/>
       <c r="P7" s="1"/>
     </row>
     <row r="8" spans="1:21" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -3255,17 +3255,17 @@
       <c r="U12"/>
     </row>
     <row r="14" spans="1:21" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C14" s="64" t="s">
+      <c r="C14" s="65" t="s">
         <v>393</v>
       </c>
-      <c r="D14" s="64"/>
-      <c r="E14" s="64"/>
-      <c r="F14" s="64"/>
-      <c r="G14" s="64"/>
-      <c r="H14" s="64"/>
-      <c r="I14" s="64"/>
-      <c r="J14" s="64"/>
-      <c r="K14" s="64"/>
+      <c r="D14" s="65"/>
+      <c r="E14" s="65"/>
+      <c r="F14" s="65"/>
+      <c r="G14" s="65"/>
+      <c r="H14" s="65"/>
+      <c r="I14" s="65"/>
+      <c r="J14" s="65"/>
+      <c r="K14" s="65"/>
       <c r="L14" s="7"/>
       <c r="M14" s="7"/>
       <c r="N14" s="1"/>
@@ -3463,19 +3463,19 @@
       </c>
     </row>
     <row r="21" spans="1:23" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C21" s="64" t="s">
+      <c r="C21" s="65" t="s">
         <v>390</v>
       </c>
-      <c r="D21" s="64"/>
-      <c r="E21" s="64"/>
-      <c r="F21" s="64"/>
-      <c r="G21" s="64"/>
-      <c r="H21" s="64"/>
-      <c r="I21" s="64"/>
-      <c r="J21" s="64"/>
-      <c r="K21" s="64"/>
-      <c r="L21" s="64"/>
-      <c r="M21" s="64"/>
+      <c r="D21" s="65"/>
+      <c r="E21" s="65"/>
+      <c r="F21" s="65"/>
+      <c r="G21" s="65"/>
+      <c r="H21" s="65"/>
+      <c r="I21" s="65"/>
+      <c r="J21" s="65"/>
+      <c r="K21" s="65"/>
+      <c r="L21" s="65"/>
+      <c r="M21" s="65"/>
       <c r="T21" s="2"/>
       <c r="U21"/>
     </row>
@@ -3734,7 +3734,7 @@
     </row>
     <row r="28" spans="1:23" x14ac:dyDescent="0.25">
       <c r="C28" s="27" t="s">
-        <v>635</v>
+        <v>636</v>
       </c>
     </row>
     <row r="29" spans="1:23" x14ac:dyDescent="0.25">

</xml_diff>